<commit_message>
Add auto-refresh & refresh button to BeritaPage
Introduce automatic and manual data refresh in Pertemuan7/src/app/page.tsx: add loadBerita(), refreshing and lastUpdated states, call loadBerita on mount and every 30s via setInterval, and show last update timestamp plus a Refresh button (disables while refreshing). Improve header layout to display update info and refresh control. Also include updates to scraping artifacts: hasil_cleaning.xlsx replaced and log_otomasi.txt appended with recent automation run entries.
</commit_message>
<xml_diff>
--- a/Pertemuan8/scraping/hasil_cleaning.xlsx
+++ b/Pertemuan8/scraping/hasil_cleaning.xlsx
@@ -460,35 +460,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Samsung Mulai Produksi Layar OLED untuk iPhone Lipat</t>
+          <t>Elon Musk Tak Lagi Triliuner, Saham SpaceX Ambles 30%</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Samsung Mulai Produksi Layar OLED untuk iPhone Lipat</t>
+          <t>Elon Musk Tak Lagi Triliuner, Saham SpaceX Ambles 30%</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8544665/samsung-mulai-produksi-layar-oled-untuk-iphone-lipat</t>
+          <t>https://inet.detik.com/cyberlife/d-8544684/elon-musk-tak-lagi-triliuner-saham-spacex-ambles-30</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://inet.detik.com/consumer/d-8544665/samsung-mulai-produksi-layar-oled-untuk-iphone-lipat</t>
+          <t>https://inet.detik.com/cyberlife/d-8544684/elon-musk-tak-lagi-triliuner-saham-spacex-ambles-30</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://awsimages.detik.net.id/community/media/visual/2025/03/07/iphone-layar-lipat-1741311565657_43.jpeg?w=250&amp;q=90</t>
+          <t>https://awsimages.detik.net.id/community/media/visual/2025/06/06/pasang-surut-hubungan-trump-elon-musk-1749210403271_43.jpeg?w=250&amp;q=90</t>
         </is>
       </c>
       <c r="F2" s="1" t="n">
-        <v>46197.48970667486</v>
+        <v>46197.52981121456</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Jakarta - Ponsel foldable pertama Apple, mungkin akan dinamai iPhone Ultra, diperkirakan akan dirilis pada September 2026 mendatang, dan kini kabarnya Samsung sudah mulai memproduksi panel OLED untuk perangkat tersebut. Pada April lalu, Samsung Display memang dikabarkan menjadi pemasok utama untuk panel OLED iPhone dengan layar lipat tersebut, setelah mencapai tingkat keberhasilan produksi yang memuaskan, yaitu mencapai 80%, demikian dikutip detikINET dari GSM Arena, Rabu (24/6/2026). Kemudian sumber yang sama menyebutkan kalau Samsung Display sudah mulai memproduksi panel tersebut di pabriknya yang berlokasi di Vietnam. Pada tahap pertama, Apple disebut memesan tiga juta unit panel OLED untuk tahun 2026 ini. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Diramal Naik, Ini Bocoran Harga iPhone 18 Pro Menariknya, ada perubahan strategi terkait spesifikasi layar yang akan digunakan. Laporan pada bulan April lalu sempat menyebutkan bahwa iPhone lipat akan menggunakan display stack seri M14 milik Samsung. Namun, laporan terbaru meralat klaim tersebut. Apple tampaknya memutuskan untuk menggunakan material luminescent yang jauh lebih baru dan canggih, yakni M16. Penggunaan panel seri M16 ini diklaim akan membawa sejumlah peningkatan signifikan bagi iPhone lipat, di antaranya: Tingkat kecerahan yang jauh lebih tinggi. Reproduksi warna yang lebih akurat dan hidup. Efisiensi daya yang lebih baik, sehingga baterai lebih awet. Masa pakai komponen layar yang lebih panjang. Sebagai pelengkap, panel OLED lipat ini juga disebut akan mengintegrasikan teknologi Color Filter on Encapsulation (CoE), sebuah inovasi yang memungkinkan layar OLED menjadi lebih tipis sekaligus mengurangi pantulan cahaya tanpa memerlukan lapisan polarizer tambahan. Apple sudah mengisyaratkan produk-produknya akan mengalami kenaikan harga akibat krisis RAM dan storage yang terus berlanjut. iPhone 18 Pro yang akan rilis paruh kedua tahun ini diramal akan menjadi salah satu produk yang harganya akan naik. Dalam wawancara dengan Wall Street Journal, CEO Apple Tim Cook tidak menyebutkan produk apa saja yang akan mengalami kenaikan harga dan kapan akan berlaku. Mengingat peluncuran iPhone 18 Pro yang tidak lama lagi, kemungkinan lini produk ini akan diumumkan dengan harga lebih tinggi. Wall Street Journal mencoba membuat estimasi harga iPhone 18 Pro berdasarkan analisis internal dan informasi dari firma riset TechInsights. Baca Juga : Serba-serbi AI di iOS 27: Fitur Tercanggihnya Cuma Jalan di iPhone 17 Pro Samsung Galaxy S26 Ultra, Worth It atau Sekadar Gimik? Samsung Galaxy S26 Ultra, Worth It atau Sekadar Gimik? (asj/afr) TAGS samsung oled iphone ultra iphone lipat LIHAT LAINNYA Tautan telah disalin</t>
+          <t>Jakarta - Gelar manusia pertama dengan kekayaan lebih dari USD 1 triliun tak bertahan lama bagi Elon Musk. Setelah sempat menembus tonggak bersejarah itu usai IPO SpaceX, kekayaan Musk kini kembali turun di bawah angka triliun dolar akibat anjloknya harga saham perusahaan roket tersebut. Berdasarkan data Bloomberg Billionaires Index, kekayaan Musk kini berada di kisaran USD 957 miliar atau sekitar Rp 15.600 triliun (kurs Rp 16.300 per dolar AS). Penurunan ini terjadi setelah saham SpaceX tertekan dalam aksi jual besar-besaran yang melanda saham teknologi global. Awal bulan ini, Musk sempat mencetak sejarah sebagai triliuner pertama di dunia. Pencapaian tersebut terjadi sesaat setelah IPO SpaceX sukses besar dan membuat valuasi perusahaan melampaui USD 2 triliun. SCROLL TO CONTINUE WITH CONTENT ADVERTISEMENT Baca Juga : Elon Musk Jadi Triliuner, Para Petinggi SpaceX Ikut Tajir Melintir Kala itu, investor ritel berbondong-bondong membeli saham SpaceX. Optimisme terhadap berbagai proyek futuristis perusahaan, mulai dari pusat data di luar angkasa hingga ambisi mengirim manusia ke Mars, mendorong harga saham melesat tajam dalam beberapa hari pertama perdagangan. Namun euforia tersebut kini mulai mereda. Saham SpaceX ditutup di level sekitar USD 156 pada perdagangan Selasa (23/6/2026), turun lebih dari 30% dibandingkan puncak intraday USD 225 yang tercapai pada 16 Juni lalu. Meski demikian, harga tersebut masih sedikit lebih tinggi dibandingkan harga debut IPO di level USD 150 per saham. Penurunan saham SpaceX terjadi di tengah koreksi yang melanda sektor teknologi. Kekhawatiran terhadap potensi gelembung (bubble) industri AI serta prospek kenaikan suku bunga membuat investor mulai mengurangi eksposur terhadap saham-saham teknologi dengan valuasi tinggi. Sejumlah analis juga mulai mempertanyakan valuasi fantastis SpaceX yang dianggap terlalu tinggi dibandingkan kondisi fundamental perusahaan saat ini. Sorotan semakin besar setelah dokumen IPO mengungkapkan bahwa SpaceX membukukan kerugian sebesar USD 4,9 miliar sepanjang 2025. SpaceX IPO Foto: Morningbrew Tak hanya itu, divisi kecerdasan buatan (AI) milik SpaceX disebut menghabiskan belanja modal hingga USD 12,7 miliar, sehingga memicu kekhawatiran soal kemampuan perusahaan menghasilkan keuntungan dalam jangka pendek. Tantangan berikutnya datang dari berakhirnya periode lockup IPO dalam beberapa bulan mendatang. Momen tersebut akan memungkinkan investor awal dan karyawan menjual saham mereka ke pasar, yang berpotensi menambah tekanan terhadap harga saham. Meski demikian, SpaceX masih menjadi aset terbesar Musk. Kepemilikan sahamnya di perusahaan tersebut diperkirakan bernilai sekitar USD 744 miliar atau hampir 80% dari total kekayaannya. Sementara kepemilikannya di Tesla juga ikut tergerus koreksi pasar dan kini bernilai sekitar USD 158 miliar. Walau kehilangan status triliuner, posisi Musk sebagai orang terkaya di dunia masih sangat aman. Jarak kekayaannya dengan pesaing terdekat, Larry Page, masih mencapai sekitar US$ 660 miliar. Sebagai gambaran, selisih tersebut bahkan lebih besar dari dua kali total kekayaan Jeff Bezos. Dengan kata lain, meski turun dari level triliuner, Musk masih berada jauh di depan para miliarder lainnya dalam daftar orang terkaya dunia. Baca Juga : Hal yang Bakal Gantikan Uang Menurut Ramalan Elon Musk Video Presiden Meksiko Geram Dikaitkan dengan Kartel Narkoba oleh Elon Musk Video Presiden Meksiko Geram Dikaitkan dengan Kartel Narkoba oleh Elon Musk (afr/afr) TAGS elon musk triliuner saham spacex ipo spacex kekayaan elon musk penurunan saham investasi teknologi pasar saham larry page LIHAT LAINNYA Tautan telah disalin</t>
         </is>
       </c>
     </row>

</xml_diff>